<commit_message>
Agregar campos opcionales para subtítulos y descripciones cortas en colecciones de Shopify y actualizar la lógica de importación para incluir estos nuevos campos.
</commit_message>
<xml_diff>
--- a/LovLory_estructura_colecciones_shopify_MVP_v1.xlsx
+++ b/LovLory_estructura_colecciones_shopify_MVP_v1.xlsx
@@ -113,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -194,6 +194,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -974,7 +980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="24" min="1" max="1"/>
@@ -988,6 +994,8 @@
     <col width="42" customWidth="1" style="24" min="9" max="9"/>
     <col width="22" customWidth="1" style="24" min="10" max="10"/>
     <col width="55" customWidth="1" style="24" min="11" max="11"/>
+    <col width="55" customWidth="1" style="24" min="12" max="12"/>
+    <col width="55" customWidth="1" style="24" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" s="24">
@@ -1006,8 +1014,13 @@
       <c r="I1" s="27" t="n"/>
       <c r="J1" s="27" t="n"/>
       <c r="K1" s="27" t="n"/>
-    </row>
-    <row r="2"/>
+      <c r="L1" s="35" t="n"/>
+      <c r="M1" s="35" t="n"/>
+    </row>
+    <row r="2">
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+    </row>
     <row r="3" ht="28" customHeight="1" s="24">
       <c r="A3" s="28" t="inlineStr">
         <is>
@@ -1064,6 +1077,16 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="L3" s="36" t="inlineStr">
+        <is>
+          <t>Subtítulo superior cabecera</t>
+        </is>
+      </c>
+      <c r="M3" s="36" t="inlineStr">
+        <is>
+          <t>Descripción corta cabecera</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="29" t="inlineStr">
@@ -1119,6 +1142,8 @@
           <t>Landing paraguas de bienestar sensorial. La clienta insiste en no tratarlo como solo 'cremas'.</t>
         </is>
       </c>
+      <c r="L4" s="37" t="inlineStr"/>
+      <c r="M4" s="37" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
@@ -1174,6 +1199,8 @@
           <t>Incluye hidratantes vulvares, elixires de placer y cuidado del suelo pélvico.</t>
         </is>
       </c>
+      <c r="L5" s="37" t="n"/>
+      <c r="M5" s="37" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
@@ -1229,6 +1256,8 @@
           <t>Seguir esquema de clienta. Útil como landing/listado si hay catálogo suficiente; tono cuidado y bienestar íntimo.</t>
         </is>
       </c>
+      <c r="L6" s="37" t="n"/>
+      <c r="M6" s="37" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
@@ -1284,6 +1313,8 @@
           <t>Subcolección propuesta por clienta. Evitar claims; enfocar en experiencia sensorial.</t>
         </is>
       </c>
+      <c r="L7" s="37" t="n"/>
+      <c r="M7" s="37" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
@@ -1339,6 +1370,8 @@
           <t>Subcolección delicada: enfoque educativo y bienestar; revisar claims de salud.</t>
         </is>
       </c>
+      <c r="L8" s="37" t="n"/>
+      <c r="M8" s="37" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
@@ -1394,6 +1427,8 @@
           <t>Incluye geles de higiene, retardantes y vigorizantes.</t>
         </is>
       </c>
+      <c r="L9" s="37" t="n"/>
+      <c r="M9" s="37" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
@@ -1449,6 +1484,8 @@
           <t>Seguir esquema de clienta. Naming sobrio y de cuidado personal.</t>
         </is>
       </c>
+      <c r="L10" s="37" t="n"/>
+      <c r="M10" s="37" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
@@ -1504,6 +1541,8 @@
           <t>Colección sensible; evitar promesas médicas o resultados garantizados.</t>
         </is>
       </c>
+      <c r="L11" s="37" t="n"/>
+      <c r="M11" s="37" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
@@ -1559,6 +1598,8 @@
           <t>Colección sensible; enfocar como bienestar/sensación, no tratamiento.</t>
         </is>
       </c>
+      <c r="L12" s="37" t="n"/>
+      <c r="M12" s="37" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
@@ -1614,6 +1655,8 @@
           <t>Nuevo bloque añadido desde el Excel de la clienta. Contiene lubricantes, geles con efectos y espumas crocanti para masaje.</t>
         </is>
       </c>
+      <c r="L13" s="37" t="n"/>
+      <c r="M13" s="37" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
@@ -1669,6 +1712,8 @@
           <t>Base agua, silicona y sabores como filtros; mantener colección por intención comercial clara.</t>
         </is>
       </c>
+      <c r="L14" s="37" t="n"/>
+      <c r="M14" s="37" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="29" t="inlineStr">
@@ -1724,6 +1769,8 @@
           <t>Cliente lo contempla como sublínea. Puede ser landing si hay suficiente producto; si no, mantener como filtro.</t>
         </is>
       </c>
+      <c r="L15" s="37" t="n"/>
+      <c r="M15" s="37" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="29" t="inlineStr">
@@ -1779,6 +1826,8 @@
           <t>Subcategoría muy específica; crear solo si hay referencias reales suficientes, pero dejar prevista por petición clienta.</t>
         </is>
       </c>
+      <c r="L16" s="37" t="n"/>
+      <c r="M16" s="37" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="29" t="inlineStr">
@@ -1834,6 +1883,8 @@
           <t>Incluye aceites esenciales, perfumes con feromonas y velas de masaje.</t>
         </is>
       </c>
+      <c r="L17" s="37" t="n"/>
+      <c r="M17" s="37" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="29" t="inlineStr">
@@ -1889,6 +1940,8 @@
           <t>Subcolección según esquema clienta. Valorar si se muestra como enlace directo o filtro si hay poco catálogo.</t>
         </is>
       </c>
+      <c r="L18" s="37" t="n"/>
+      <c r="M18" s="37" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="29" t="inlineStr">
@@ -1944,6 +1997,8 @@
           <t>Revisar claims de feromonas en contenido; evitar promesas no demostrables.</t>
         </is>
       </c>
+      <c r="L19" s="37" t="n"/>
+      <c r="M19" s="37" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="29" t="inlineStr">
@@ -1999,6 +2054,8 @@
           <t>Buena colección para regalo y venta cruzada con parejas/packs.</t>
         </is>
       </c>
+      <c r="L20" s="37" t="n"/>
+      <c r="M20" s="37" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="29" t="inlineStr">
@@ -2054,6 +2111,8 @@
           <t>Landing paraguas de tecnología y placer.</t>
         </is>
       </c>
+      <c r="L21" s="37" t="n"/>
+      <c r="M21" s="37" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="29" t="inlineStr">
@@ -2109,6 +2168,8 @@
           <t>Una de las colecciones con más intención comercial.</t>
         </is>
       </c>
+      <c r="L22" s="37" t="n"/>
+      <c r="M22" s="37" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="29" t="inlineStr">
@@ -2164,6 +2225,8 @@
           <t>Útil para tono de bienestar/pareja.</t>
         </is>
       </c>
+      <c r="L23" s="37" t="n"/>
+      <c r="M23" s="37" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="29" t="inlineStr">
@@ -2219,6 +2282,8 @@
           <t>Nombrar con enfoque salud, iniciación y seguridad.</t>
         </is>
       </c>
+      <c r="L24" s="37" t="n"/>
+      <c r="M24" s="37" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="29" t="inlineStr">
@@ -2274,6 +2339,8 @@
           <t>Muy útil para primeras compras y recomendaciones.</t>
         </is>
       </c>
+      <c r="L25" s="37" t="n"/>
+      <c r="M25" s="37" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="29" t="inlineStr">
@@ -2329,6 +2396,8 @@
           <t>Aquí encajan productos tipo Mistress.</t>
         </is>
       </c>
+      <c r="L26" s="37" t="n"/>
+      <c r="M26" s="37" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="29" t="inlineStr">
@@ -2384,6 +2453,8 @@
           <t>Mencionadas por clienta; valorar visibilidad por sensibilidad/stock.</t>
         </is>
       </c>
+      <c r="L27" s="37" t="n"/>
+      <c r="M27" s="37" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="29" t="inlineStr">
@@ -2439,6 +2510,8 @@
           <t>Misma lógica que muñecas tamaño real.</t>
         </is>
       </c>
+      <c r="L28" s="37" t="n"/>
+      <c r="M28" s="37" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="29" t="inlineStr">
@@ -2494,6 +2567,8 @@
           <t>Landing paraguas para moda íntima.</t>
         </is>
       </c>
+      <c r="L29" s="37" t="n"/>
+      <c r="M29" s="37" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="29" t="inlineStr">
@@ -2549,6 +2624,8 @@
           <t>Mapalé/Mapelé se ubica aquí. En el Excel de clienta se menciona especialmente 'Conjuntos'.</t>
         </is>
       </c>
+      <c r="L30" s="37" t="n"/>
+      <c r="M30" s="37" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="29" t="inlineStr">
@@ -2604,6 +2681,8 @@
           <t>Fetish Submissive se ubica aquí. Cuero, vinilo, arneses y lencería sado como filtros/metafields.</t>
         </is>
       </c>
+      <c r="L31" s="37" t="n"/>
+      <c r="M31" s="37" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="29" t="inlineStr">
@@ -2659,6 +2738,8 @@
           <t>Muy relevante por CSV Mapalé/Ensemble Sexy y por comentario explícito de la clienta.</t>
         </is>
       </c>
+      <c r="L32" s="37" t="n"/>
+      <c r="M32" s="37" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="29" t="inlineStr">
@@ -2714,6 +2795,8 @@
           <t>Relevante por CSV Mapalé/Bodys, aunque no aparece como sublínea explícita en el Excel de la clienta.</t>
         </is>
       </c>
+      <c r="L33" s="37" t="n"/>
+      <c r="M33" s="37" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="29" t="inlineStr">
@@ -2769,6 +2852,8 @@
           <t>Unificar Nuisettes &amp; Babydolls/Nuisette del proveedor.</t>
         </is>
       </c>
+      <c r="L34" s="37" t="n"/>
+      <c r="M34" s="37" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="29" t="inlineStr">
@@ -2824,6 +2909,8 @@
           <t>Medias, pezoneras y antifaces. Antifaces pueden aparecer también vinculados a BDSM si aplica.</t>
         </is>
       </c>
+      <c r="L35" s="37" t="n"/>
+      <c r="M35" s="37" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="29" t="inlineStr">
@@ -2879,6 +2966,8 @@
           <t>Separar hardware BDSM de lencería fetish.</t>
         </is>
       </c>
+      <c r="L36" s="37" t="n"/>
+      <c r="M36" s="37" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="29" t="inlineStr">
@@ -2934,6 +3023,8 @@
           <t>Incluye esposas, cuerdas, arneses de cama y columpios según Excel de clienta.</t>
         </is>
       </c>
+      <c r="L37" s="37" t="n"/>
+      <c r="M37" s="37" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="29" t="inlineStr">
@@ -2989,6 +3080,8 @@
           <t>Látigos, palas, plumas y fustas.</t>
         </is>
       </c>
+      <c r="L38" s="37" t="n"/>
+      <c r="M38" s="37" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="29" t="inlineStr">
@@ -3044,6 +3137,8 @@
           <t>Categoría sensible; naming sobrio.</t>
         </is>
       </c>
+      <c r="L39" s="37" t="n"/>
+      <c r="M39" s="37" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="29" t="inlineStr">
@@ -3099,6 +3194,8 @@
           <t>Landing lúdica y de regalo.</t>
         </is>
       </c>
+      <c r="L40" s="37" t="n"/>
+      <c r="M40" s="37" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="29" t="inlineStr">
@@ -3154,6 +3251,8 @@
           <t>Cartas de retos, dados eróticos y juegos de rol.</t>
         </is>
       </c>
+      <c r="L41" s="37" t="n"/>
+      <c r="M41" s="37" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="29" t="inlineStr">
@@ -3209,6 +3308,8 @@
           <t>Cajas cerradas temáticas y cestas personalizables.</t>
         </is>
       </c>
+      <c r="L42" s="37" t="n"/>
+      <c r="M42" s="37" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3224,7 +3325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="24" min="1" max="1"/>
@@ -3237,6 +3338,8 @@
     <col width="16" customWidth="1" style="24" min="8" max="8"/>
     <col width="14" customWidth="1" style="24" min="9" max="9"/>
     <col width="58" customWidth="1" style="24" min="10" max="10"/>
+    <col width="58" customWidth="1" style="24" min="11" max="11"/>
+    <col width="58" customWidth="1" style="24" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" s="24">
@@ -3254,8 +3357,13 @@
       <c r="H1" s="6" t="n"/>
       <c r="I1" s="6" t="n"/>
       <c r="J1" s="6" t="n"/>
-    </row>
-    <row r="2"/>
+      <c r="K1" s="11" t="n"/>
+      <c r="L1" s="11" t="n"/>
+    </row>
+    <row r="2">
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+    </row>
     <row r="3" ht="24" customHeight="1" s="24">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -3307,6 +3415,16 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="K3" s="21" t="inlineStr">
+        <is>
+          <t>Subtítulo superior cabecera</t>
+        </is>
+      </c>
+      <c r="L3" s="21" t="inlineStr">
+        <is>
+          <t>Descripción corta cabecera</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
@@ -3359,6 +3477,8 @@
           <t>Crear como colección viva. Shopify no siempre replica 'últimos añadidos' por fecha como regla automática; lo más fiable es taggear novedades en importación/publicación y retirar el tag cuando deje de ser novedad.</t>
         </is>
       </c>
+      <c r="K4" s="23" t="inlineStr"/>
+      <c r="L4" s="23" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="22" t="inlineStr">
@@ -3411,6 +3531,8 @@
           <t>Crear colección propia para home, menú, SEO y campañas. También puede existir filtro de descuento dentro de categorías, pero no sustituye la landing de Ofertas.</t>
         </is>
       </c>
+      <c r="K5" s="23" t="n"/>
+      <c r="L5" s="23" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3426,7 +3548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="24" min="1" max="1"/>
@@ -3436,6 +3558,8 @@
     <col width="44" customWidth="1" style="24" min="5" max="5"/>
     <col width="38" customWidth="1" style="24" min="6" max="6"/>
     <col width="58" customWidth="1" style="24" min="7" max="7"/>
+    <col width="58" customWidth="1" style="24" min="8" max="8"/>
+    <col width="58" customWidth="1" style="24" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" s="24">
@@ -3450,8 +3574,13 @@
       <c r="E1" s="6" t="n"/>
       <c r="F1" s="6" t="n"/>
       <c r="G1" s="6" t="n"/>
-    </row>
-    <row r="2"/>
+      <c r="H1" s="11" t="n"/>
+      <c r="I1" s="11" t="n"/>
+    </row>
+    <row r="2">
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+    </row>
     <row r="3" ht="24" customHeight="1" s="24">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -3488,6 +3617,16 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="H3" s="21" t="inlineStr">
+        <is>
+          <t>Subtítulo superior cabecera</t>
+        </is>
+      </c>
+      <c r="I3" s="21" t="inlineStr">
+        <is>
+          <t>Descripción corta cabecera</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
@@ -3525,6 +3664,8 @@
           <t>Marca indicada por clienta como cosmética íntima.</t>
         </is>
       </c>
+      <c r="H4" s="23" t="inlineStr"/>
+      <c r="I4" s="23" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="22" t="inlineStr">
@@ -3562,6 +3703,8 @@
           <t>Marca premium/tecnología unisex.</t>
         </is>
       </c>
+      <c r="H5" s="23" t="n"/>
+      <c r="I5" s="23" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="22" t="inlineStr">
@@ -3599,6 +3742,8 @@
           <t>Bienestar masculino y masturbadores.</t>
         </is>
       </c>
+      <c r="H6" s="23" t="n"/>
+      <c r="I6" s="23" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="22" t="inlineStr">
@@ -3636,6 +3781,8 @@
           <t>Clienta indica que ya está en web vieja.</t>
         </is>
       </c>
+      <c r="H7" s="23" t="n"/>
+      <c r="I7" s="23" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5395,7 +5542,7 @@
           <t>MVP Shopify</t>
         </is>
       </c>
-      <c r="B17" s="35" t="inlineStr">
+      <c r="B17" s="37" t="inlineStr">
         <is>
           <t>Se crean principales; secundarias solo Novedades y Ofertas; marcas ORGIE, SVAKOM, TENGA y MISTRESS.</t>
         </is>
@@ -5410,7 +5557,7 @@
           <t>Documento MVP v1 generado para ejecución inicial en Shopify.</t>
         </is>
       </c>
-      <c r="E17" s="35" t="inlineStr">
+      <c r="E17" s="37" t="inlineStr">
         <is>
           <t>Pendiente validar exportación real de productos y taxonomía limpia de tags/metafields.</t>
         </is>

</xml_diff>